<commit_message>
Refresh first twenty ratings and add dashboard videos
</commit_message>
<xml_diff>
--- a/rating-results.xlsx
+++ b/rating-results.xlsx
@@ -259,161 +259,161 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c>
-        <v>0.857</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is quite abstract and could be interpreted as waving, signaling, or pointing rather than specifically representing a traffic light.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture represents 'stop' rather than the object 'traffic light' itself, which might cause slight confusion if learners expect a representation of the three lights.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is abstract and does not clearly depict the physical structure or function of a traffic light.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture visually represents the action of stopping rather than the physical shape or appearance of a traffic light, making the visual resemblance to the object itself weak.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>There is a slight action-related element, but it does not strongly evoke the experience of interacting with a traffic light.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture evokes the physical action of halting or directing traffic, providing a moderate bodily connection to the function of a traffic light.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and lacks distinct emotional or dynamic emphasis.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is straightforward and functional, lacking significant dynamic emphasis or emotional expressiveness.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
+          <t>high</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c>
+        <v>0.286</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could potentially be interpreted as a generic 'stop' signal or a 'wait' gesture if not contextualized.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture signifies 'stop' rather than the physical object 'traffic light', which might be slightly ambiguous without context.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>-1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The vertical movement of the hand clearly mimics the sequence of a traffic light changing colors.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture represents the 'stop' command associated with a red traffic light, rather than the physical appearance of the light itself.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>It simulates the visual experience of observing a traffic light, though it lacks the physical interaction of driving.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Evokes the physical action of halting or signaling someone to stop, which is the primary function of a traffic light.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, though not particularly expansive or rapid.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is a clear, deliberate raising of the arm, moderate in size and speed.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
+        </is>
       </c>
       <c t="inlineStr">
         <is>
           <t>The actor maintains a neutral facial expression throughout the gesture.</t>
         </is>
       </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral facial expression throughout the gesture, providing no emotional cues.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple and easy to perform, though its connection to the target word is weak.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is extremely simple and clear, making it an optimal, low-cognitive-load movement for a learning context.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is not a standard or widely recognized cultural sign for a traffic light.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The raised open palm is a universally recognized gesture for 'stop', which is strongly associated with traffic control.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very simple and physically easy for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement involves a basic arm raise and hand position that is effortless for learners to reproduce.</t>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly suited for representing the concept of a traffic light.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is very simple, direct, and perfectly balances informativeness with ease of understanding.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Traffic lights are a universal cultural symbol, and the vertical motion is widely understood.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The raised hand with palm facing outward is a highly familiar and universally recognized sign for 'stop' in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very simple and easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture involves a basic arm movement that is effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -447,57 +447,57 @@
         </is>
       </c>
       <c>
-        <v>0.286</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture could potentially be interpreted as 'hitching' or 'towing' generally, rather than specifically 'trailer'.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture represents the action associated with the object (pulling) rather than the shape of the object itself, which could be interpreted as 'pull' or 'tow'.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture mimics the physical action of hitching a trailer to a vehicle, which is a clear iconic representation of the word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture clearly represents the defining function of a trailer, which is being pulled behind a vehicle or person.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement simulates the specific physical interaction of connecting a trailer, engaging the body in a functional task.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The forward lean and backward arm extension strongly simulate the physical effort and bodily experience of towing a heavy load.</t>
+        <v>0.714</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could be interpreted as hitching a trailer, but without context, it might also look like simply reaching behind one's back.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture represents the action of pulling rather than the object itself, which could be interpreted as verbs like 'pull' or 'drag'.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture mimics the act of hitching a trailer to a vehicle, which is a moderate iconic representation of the word's function.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture clearly depicts the action of towing or pulling something behind, which is the defining characteristic of a trailer.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>It simulates the physical action of connecting a trailer, providing a moderate sensorimotor link to the concept.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The posture and arm position strongly evoke the physical sensation of dragging or pulling a heavy load.</t>
         </is>
       </c>
       <c>
@@ -511,12 +511,12 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is functional and precise but lacks significant emotional intensity or dynamic emphasis.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is deliberate and conveys physical effort, but lacks strong emotional expressiveness.</t>
+          <t>The movement is relatively small and constrained to the area behind the back, making it somewhat subtle.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement involves a full-body shift and arm extension, making it moderately salient but not overly expansive.</t>
         </is>
       </c>
       <c>
@@ -530,69 +530,69 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The actor maintains a neutral, task-focused facial expression throughout the gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's facial expression remains mostly neutral, with only a slight indication of focus or effort while looking back.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly suited for illustrating the concept of a trailer.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and effectively conveys the core concept without unnecessary complexity.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of hitching a trailer is a widely understood mechanical concept in many cultures.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The pantomime of pulling something heavy behind oneself is a widely understood concept across cultures.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is very simple and involves basic arm and torso movements that are easy for anyone to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement involves basic body mechanics that are very easy for learners to reproduce.</t>
+          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The facial expression is mostly neutral, showing only a slight hint of physical effort.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, clear, and directly related to the concept without unnecessary complexity.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is straightforward and effectively conveys the concept without unnecessary complexity.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of hitching a trailer is a recognizable concept in many Western contexts, though the specific gesture is not a standard emblem.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Pantomiming pulling something behind oneself is a recognizable way to represent towing or a trailer.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very simple and easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is simple, requires no special coordination, and is very easy for learners to enact.</t>
         </is>
       </c>
     </row>
@@ -633,107 +633,107 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture could also be interpreted as leaning on a fence or a counter, but in the context of 'balcony', it is highly appropriate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Without the target word, the gesture could potentially be interpreted as leaning on a fence, a counter, or looking out a window.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The posture of leaning on an imaginary railing is a clear and recognizable representation of standing on a balcony.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture clearly represents the action of leaning on a railing, which is strongly associated with a balcony, depicting the interaction with the object rather than the architectural structure itself.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture effectively simulates the physical experience of leaning on a balcony railing.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture vividly simulates the physical action and bodily posture of resting one's arms on a balcony railing.</t>
-        </is>
+          <t>The gesture could potentially be interpreted as leaning on a fence or a counter, but in the context of the word 'balcony', it is highly specific.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could potentially be interpreted as leaning on a table or a fence, though 'balcony' is a very strong fit.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The posture of leaning on an imaginary railing is a clear and recognizable iconic representation of standing on a balcony.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture clearly depicts the action of leaning on a railing, visually representing the physical structure and typical interaction with a balcony.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture effectively simulates the physical experience of leaning on a balcony railing, engaging the upper body in a way that mirrors the real-world action.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture strongly evokes the bodily experience of resting one's arms on a solid surface and leaning forward to look out.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and purposeful, though relatively contained and static, which is appropriate for the nature of the action being depicted.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, but moderate in its spatial extent and speed.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c>
         <v>2</v>
       </c>
       <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and descriptive rather than emotionally expressive.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is calm, smooth, and deliberate, lacking strong emotional dynamics or intensity.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's facial expression remains neutral throughout the gesture.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, intuitive, and perfectly suited for representing the concept of a balcony.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly balances informativeness with ease of understanding for a learner.</t>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor's facial expression remains mostly neutral, with only a slight indication of looking outward.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly suited for representing the concept of a balcony without unnecessary complexity.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, direct, and optimally balances informativeness with ease of understanding for a learner.</t>
         </is>
       </c>
       <c>
@@ -747,31 +747,31 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>Leaning on a railing is a universally understood posture associated with balconies.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of leaning on a railing is a common and widely recognized behavior across many cultures.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is very simple and natural for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture involves a simple arm movement and a slight body lean that is effortless for anyone to reproduce.</t>
+          <t>The action of leaning on a railing is a universally understood gesture in Western contexts.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Pantomiming leaning on a railing is a common and easily understood way to represent a balcony or looking out from a height in Western culture.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is very simple and natural, making it extremely easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very natural, requires no special coordination, and is effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -805,152 +805,152 @@
         </is>
       </c>
       <c>
-        <v>0.571</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture could also represent 'round', 'circle', or 'throwing' depending on context.</t>
-        </is>
+        <v>0.143</v>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The curved arm movement clearly mimics the round shape of a ball.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture clearly depicts the shape of the object and the primary action associated with it (throwing), making it highly transparent.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement simulates the physical interaction of holding or shaping a spherical object.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of gripping an imaginary object and performing a throwing motion provides a very vivid bodily experience related to a ball.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and descriptive rather than emotionally expressive.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement has a clear trajectory and dynamic emphasis during the throw, but it is functional rather than emotionally expressive.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral, task-oriented facial expression throughout.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's facial expression remains largely neutral, with only a slight look of focus during the throwing action.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly suited for representing the concept of a ball.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The two-part motion (holding, then throwing) is simple, intuitive, and perfectly captures the concept without being overloaded.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using hands to indicate a round shape is a universal gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of holding and throwing a ball is a universally recognized physical activity across cultures.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very simple and easy for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very natural, requires no special coordination, and is effortless for learners to mimic.</t>
+      <c t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The circular hand movement clearly and transparently depicts the spherical shape of a ball.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The hands forming a spherical shape combined with a throwing motion provides a highly transparent visual representation of a ball and its typical use.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture simulates the physical interaction of tracing the outline of a round object, evoking the tactile experience of a ball.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture vividly simulates the physical sensation of holding a round object and the bodily action of throwing it.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is expansive and uses both arms, making it visually prominent and easy to follow.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture involves a clear, expansive movement of both arms across and away from the body, making it visually prominent.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor's facial expression remains neutral throughout the gesture, conveying no affective meaning.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly suited for representing the concept of a ball.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is straightforward and perfectly balances simplicity with clear semantic meaning, making it optimal for learning.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Tracing a circle to represent a round object is a universally understood and highly familiar gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The pantomime of holding and throwing a ball is a highly recognizable and universally understood action in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is very simple and natural, making it extremely easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The throwing motion is very natural, requires no special coordination, and is effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -984,21 +984,21 @@
         </is>
       </c>
       <c>
-        <v>0.0</v>
-      </c>
-      <c>
-        <v>0</v>
+        <v>0.143</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could also be interpreted as 'sleep' or 'tired' rather than specifically 'bed', though it is strongly associated with the object.</t>
+        </is>
       </c>
       <c t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c>
         <v>5</v>
       </c>
@@ -1015,121 +1015,121 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is a highly transparent metonymic representation, using the action of sleeping to clearly indicate the object 'bed'.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>It directly simulates the physical posture and sensation of resting one's head on a pillow, evoking the sensorimotor experience of sleeping.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture directly and vividly simulates the physical bodily experience of resting one's head on a pillow.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is smooth and deliberate, effectively conveying the calm associated with sleep, though it is not highly dynamic.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is slow, gentle, and calming, which perfectly fits the concept of rest, though it lacks high dynamic intensity.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor adopts a soft, relaxed facial expression with closed eyes, which clearly communicates the state of sleepiness or rest.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's closed eyes and relaxed facial expression clearly communicate a peaceful and restful affective state.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, intuitive, and perfectly suited for vocabulary learning as it is easy to associate with the target word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is extremely simple, intuitive, and perfectly balances informativeness with ease of cognitive processing.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The 'hands-under-cheek' gesture for sleeping is a cross-culturally recognized symbol.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Resting the head on folded hands is a universally recognized and highly familiar gesture for sleep or a bed.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is very simple and natural, making it extremely easy for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture requires minimal motor coordination and is effortless for learners to reproduce.</t>
+          <t>The gesture of resting the head on folded hands perfectly mimics the action of sleeping on a pillow, strongly representing the concept of a bed.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>It directly simulates the physical posture and sensation of resting one's head on a pillow, evoking the bodily experience of sleeping.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture directly simulates the bodily experience of resting the head, evoking strong sensorimotor associations with lying in a bed.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, though relatively small and contained within the upper body space.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is smooth and constrained to the upper body, lacking large or rapid dynamics.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>-1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor adopts a calm, closed-eye expression that effectively conveys the feeling of sleepiness or relaxation.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor's face relaxes and eyes close slightly, conveying a calm, restful state associated with sleeping.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly suited for learners of all levels.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and easy to process, making it ideal for learning.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The 'hands-under-cheek' gesture for sleeping is a highly common and culturally universal signifier.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Placing hands together under a tilted head is a widely recognized emblem for sleep in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is extremely easy and natural for anyone to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is simple, requires no special coordination, and is effortless to perform.</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>Could potentially be interpreted as 'frame', 'picture', or 'window' depending on context.</t>
+          <t>The gesture could potentially be interpreted as 'frame', 'picture', or 'television' depending on context, though 'monitor' is the most logical fit.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -1189,64 +1189,64 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The rectangular hand shape clearly mimics the frame of a computer monitor or screen.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture directly traces the physical, rectangular shape of a monitor, providing a highly transparent visual representation of the object.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>It simulates the act of framing or looking at a screen, which is a common perceptual experience associated with the word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action involves tracing an outline, which evokes the physical dimensions of the object, but it does not simulate interacting with or using a monitor.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and precise rather than emotionally expressive.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is smooth, deliberate, and descriptive, lacking strong emotional dynamics or intensity.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral, task-oriented facial expression throughout.</t>
+          <t>The gesture clearly outlines the rectangular shape of a monitor screen, making the iconic relationship to the target word very transparent.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture directly traces the rectangular shape of a computer monitor, providing a highly transparent visual representation of the object.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>It simulates the physical act of framing or defining the boundaries of a screen, which provides a moderate level of sensorimotor engagement.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of tracing the outline evokes the physical dimensions and boundaries of the object, providing moderate sensorimotor engagement.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, though not overly expansive or rapid, providing a moderate level of visual salience.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and uses both arms to draw a distinct shape in the space in front of the body, making it moderately salient.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -1265,50 +1265,50 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is simple, intuitive, and directly maps to the concept of a screen.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The simple tracing motion is optimal for conveying the concept clearly without any unnecessary motor or cognitive complexity.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using hands to frame a view or screen is a universally understood gesture in modern digital culture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Tracing a rectangle in the air to indicate a screen, picture, or monitor is a highly familiar and widely understood gesture.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is very easy to replicate and requires no special coordination.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very straightforward and effortless for learners to reproduce.</t>
+          <t>The gesture is simple, direct, and perfectly aligned with the concept of a monitor, making it highly appropriate for learning.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The simple tracing motion is perfectly balanced, conveying the meaning clearly without any unnecessary complexity.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Tracing a rectangle to represent a screen is a universally understood gesture in modern, technology-driven cultures.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Drawing a rectangle in the air is a widely recognized and common gesture for a screen, TV, or monitor in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is very simple and requires no special motor skills, making it extremely easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is simple, symmetrical, and effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture could potentially be interpreted as opening a small door or a slot for any purpose, not necessarily a letter box.</t>
+          <t>The rectangular shape could potentially be interpreted as a window or a picture frame, but the downward insertion motion clarifies the 'letter box' meaning.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -1361,71 +1361,71 @@
         <v>4</v>
       </c>
       <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The hand movements clearly simulate the physical interaction of opening a letter box slot and inserting mail.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture highly transparently represents the action of opening a letterbox and inserting mail.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture effectively simulates the tactile experience of manipulating a letter box flap.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Strongly evokes the physical sensation of holding a flap open and sliding an object into a slot.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and precise, but lacks significant emotional or dynamic intensity.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and deliberate, lacking strong emotional expressiveness.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The rectangular hand shape clearly outlines the frame of a letter box, and the downward motion mimics the act of inserting mail.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture clearly depicts the action of interacting with a letter box by simulating the insertion of a letter into a slot.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture simulates the physical interaction of placing a letter into a slot, which is a common sensorimotor experience.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture vividly evokes the physical action and bodily experience of posting a letter.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, though not overly expansive or rapid.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and pronounced, involving both arms to create a distinct action sequence.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
         </is>
       </c>
       <c t="inlineStr">
@@ -1437,57 +1437,57 @@
         <v>5</v>
       </c>
       <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>-1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly suited for representing the target word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The two-handed, asymmetrical movement is slightly complex but perfectly captures the meaning without being overwhelming.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of posting a letter is a widely understood cultural practice, though physical letter boxes are becoming less common in some digital-first societies.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of mailing a letter through a slot is a widely recognized concept across many cultures.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is very simple and involves natural hand movements that are easy for anyone to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is straightforward and easy for learners to physically reproduce.</t>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly matches the concept of a letter box.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is straightforward and perfectly balances informativeness with simplicity for learning.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The concept of a letter box and the action of posting mail are widely understood in Western cultural contexts.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of posting a letter into a slot is a highly familiar and universally understood concept in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is very simple and easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture involves simple, everyday arm movements that are very natural and effortless to reproduce.</t>
         </is>
       </c>
     </row>
@@ -1521,10 +1521,10 @@
         </is>
       </c>
       <c>
-        <v>0.0</v>
-      </c>
-      <c>
-        <v>0</v>
+        <v>0.286</v>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c t="inlineStr">
         <is>
@@ -1547,126 +1547,126 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture clearly and directly mimics the flat, overhead nature of a ceiling.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture of forming a flat surface above the head is a highly transparent visual representation of a ceiling.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>It simulates the spatial experience of reaching toward or indicating the height of a ceiling.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Reaching upwards to define a spatial boundary strongly evokes the physical experience of a ceiling's location and shape.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and clear, but lacks significant emotional or dynamic intensity.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is deliberate and descriptive, lacking strong emotional dynamics or expressive intensity.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral, task-oriented facial expression throughout.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's facial expression remains neutral throughout the video, conveying no emotional meaning.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, intuitive, and perfectly suited for learning the word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly captures the concept without any unnecessary complexity.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using hands to indicate an overhead surface is a universally understood gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using flat hands above the head to indicate a roof or ceiling is a widely recognized and common spatial gesture.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very simple and easy for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement involves a simple raising of the arms, making it very natural and effortless for learners to reproduce.</t>
+          <t>The gesture clearly and directly represents the concept of a ceiling by using the hands to define a flat, overhead boundary.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The flat hands held above the head perfectly mimic the flat, horizontal surface of a ceiling.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement simulates the physical act of reaching toward or indicating the overhead space, which is a common spatial interaction.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Reaching up and indicating the space above evokes the physical relationship and spatial awareness one has with a ceiling.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, though it is relatively simple and contained within a vertical plane.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture involves a large, upward movement of both arms, making it visually prominent and expansive.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral facial expression throughout the gesture, with no emotional cues.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, intuitive, and perfectly suited for learning the spatial concept of a ceiling.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is simple, direct, and easy to process, making it an optimal fit for vocabulary learning.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>-1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Using hands to indicate an overhead surface is a universally understood iconic gesture in Western contexts.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Indicating a flat surface above the head is a commonly understood way to represent a ceiling or roof.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture involves basic arm movements that are very easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture requires only basic motor skills (raising arms) and is effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -1707,145 +1707,145 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture could also be interpreted as representing 'arch', 'sky', or 'growth' depending on the context.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture could also represent 'tall', 'building', or 'sky', but fits 'monument' well in context.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The upward sweeping arm movement effectively traces the outline of a tall, arched, or structured monument.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The upward arm movement and gaze clearly represent the height and scale typical of a monument.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement simulates the physical scale and verticality associated with a large structure, though it lacks interaction with a specific object.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture strongly evokes the physical sensation of standing at the base of a large structure and looking up at it.</t>
-        </is>
+          <t>The gesture could potentially be interpreted as 'arch', 'building', or 'tall' without the context of the word 'monument'.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The arm movement clearly traces the outline of an arch or a tall, structured object, which is a common iconic representation of a monument.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture clearly represents the verticality and large scale typical of a monument by tracing a tall shape in the air.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture simulates the physical act of building or tracing the height and shape of a structure, engaging the upper body.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of looking up and reaching high strongly evokes the physical experience of standing at the base of a large structure.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is deliberate and expansive, though performed at a slow, steady pace.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is expansive, involving full arm extension above the head and a noticeable change in head posture.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c>
         <v>2</v>
       </c>
       <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is slow and deliberate, which conveys a sense of grandeur or stability, but it is not highly emotionally expressive.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The slow, expansive upward movement conveys a moderate sense of size and grandeur.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor's facial expression remains neutral throughout the gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The facial expression is mostly neutral, though the upward gaze suggests looking at something impressive.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, clear, and easy to associate with the concept of a large, standing structure.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and perfectly captures the core concept of a tall structure without unnecessary complexity.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using arms to represent height or a large structure is a fairly universal and intuitive gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>Using vertical space and an upward gaze to indicate height or grandeur is a widely understood concept.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very simple and involves basic arm extensions that any learner can easily replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture requires minimal coordination and is very easy for learners to reproduce.</t>
+        <v>1</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral, focused facial expression throughout the gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The facial expression is mostly neutral, though the upward gaze slightly suggests looking at something grand.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, clear, and directly maps to the concept of a tall, static structure.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, direct, and effectively conveys the core physical attribute of the target word without unnecessary complexity.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Using hands to outline the shape of a structure is a universally understood iconic gesture.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>Using upward reaching and gazing to indicate something tall or grand is a widely understood convention.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very simple and requires no special coordination, making it easy for anyone to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very natural, requires no special coordination, and is effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -1879,152 +1879,152 @@
         </is>
       </c>
       <c>
-        <v>0.429</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture could also be interpreted as 'waving' or 'sweeping' if not contextualized by the target word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture represents the action of using the ticket rather than the physical shape of the ticket itself, but the meaning remains clear.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The sweeping motion mimics the act of scanning a ticket or passing through a turnstile, which is moderately iconic for the concept of an entrance ticket.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture clearly depicts the action of handing over a small object, which strongly represents the functional use of an entrance ticket.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture simulates the physical action of presenting a ticket, engaging the arm and shoulder in a way that mimics the interaction with an entry point.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement effectively evokes the physical sensation of holding a small piece of paper and extending the arm to present it.</t>
-        </is>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>2</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is functional and clear but lacks significant emotional intensity or dynamic variation.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is deliberate and functional, lacking strong emotional dynamics or expressive intensity.</t>
-        </is>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral, task-oriented facial expression throughout the gesture.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The gesture is simple, direct, and easy to understand in the context of the target word.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The single, straightforward motion is simple to process and perfectly balanced for learning.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>1</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of scanning or presenting a ticket is a common, globally recognized experience.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The action of presenting a ticket or pass for entry is a widely recognized and common behavior.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>0</v>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The movement is very simple and requires no special coordination, making it easy for any learner to replicate.</t>
-        </is>
-      </c>
-      <c t="inlineStr">
-        <is>
-          <t>The simple arm extension and basic hand shape are effortless for learners to reproduce.</t>
+        <v>0.0</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could also be interpreted as swiping a credit card or waving a hand, but in the context of 'entrance ticket', it is highly coherent.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture could be interpreted as handing over any small object, not exclusively an entrance ticket, though the context makes it clear.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The sweeping motion effectively mimics the action of scanning a ticket or passing through an automated turnstile, which is a clear iconic representation of using an entrance ticket.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture clearly visually represents the action of presenting a ticket for entry, which is strongly associated with the target word.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture simulates the physical interaction of presenting a ticket to a scanner, engaging the arm and hand in a way that mirrors the real-world action.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture strongly evokes the physical action and bodily experience of holding a small piece of paper and handing it over.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and purposeful, though it is relatively contained and not overly expansive or rapid.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is clear and deliberate, but relatively simple and constrained to a single arm extension.</t>
+        </is>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>1</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral facial expression throughout the gesture, providing no additional affective context.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The actor maintains a neutral facial expression throughout the gesture, providing no emotional cues.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, direct, and perfectly suited for representing the concept of an entrance ticket without unnecessary cognitive load.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The gesture is simple, direct, and optimally balances informativeness with ease of understanding for a learner.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of scanning a ticket or passing through a gate is a universally recognized experience in modern Western contexts.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The action of presenting a ticket or pass is a highly familiar and universally understood convention in Western cultures.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is very simple and natural, making it extremely easy for any learner to replicate.</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>The movement is a basic, everyday arm extension that is very natural and effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture highly transparently represents the action of holding and using a remote control.</t>
+          <t>The gesture highly transparently represents the semantics by mimicking the exact action of holding and using a remote control.</t>
         </is>
       </c>
       <c>
@@ -2645,7 +2645,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture vividly simulates the physical grip and specific thumb action used to operate a remote control.</t>
+          <t>The gesture provides a very vivid simulation of the physical experience of gripping a remote and pressing a button with the thumb.</t>
         </is>
       </c>
       <c>
@@ -2664,7 +2664,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is relatively subtle, consisting only of a slight arm raise and a small thumb press.</t>
+          <t>The movement is relatively subtle and constrained, involving only a slight arm raise and a small thumb action.</t>
         </is>
       </c>
       <c>
@@ -2702,7 +2702,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is simple, direct, and perfectly captures the essence of the object without any unnecessary complexity.</t>
+          <t>The gesture is simple, direct, and perfectly captures the essence of the target word without any unnecessary complexity.</t>
         </is>
       </c>
       <c>
@@ -2721,7 +2721,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The action of pointing a handheld device and pressing a button with the thumb is universally recognized in Western cultures as using a remote control.</t>
+          <t>This pantomime of using a remote control is a highly familiar and universally understood gesture in Western cultures.</t>
         </is>
       </c>
       <c>
@@ -2740,7 +2740,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture involves minimal, everyday movements that are effortless for learners to reproduce.</t>
+          <t>The gesture involves minimal, everyday movements that are extremely natural and effortless for anyone to reproduce.</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c>
-        <v>0.143</v>
+        <v>0.286</v>
       </c>
       <c>
         <v>1</v>
@@ -2984,17 +2984,17 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The extended arms perfectly represent the wings of an airplane, and the tilting motion clearly depicts the plane banking or turning in flight.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
+          <t>Extending the arms horizontally and tilting the torso perfectly mimics the wings and banking motion of an airplane, providing a highly transparent visual representation.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c t="inlineStr">
         <is>
@@ -3003,7 +3003,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture strongly evokes the physical sensation of pretending to fly, engaging the arms and torso in a sweeping motion.</t>
+          <t>The gesture involves full upper-body engagement, vividly simulating the physical action and experience of an airplane flying and banking.</t>
         </is>
       </c>
       <c>
@@ -3022,7 +3022,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is expansive, utilizing the full wingspan of the arms and noticeable torso tilting, making it visually prominent.</t>
+          <t>The gesture involves wide arm extensions and noticeable torso tilting, making it a pronounced and expansive movement that easily captures attention.</t>
         </is>
       </c>
       <c>
@@ -3041,7 +3041,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The actor maintains a neutral facial expression throughout the gesture.</t>
+          <t>The actor maintains a neutral facial expression throughout the gesture, providing no emotional cues.</t>
         </is>
       </c>
       <c>
@@ -3060,7 +3060,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is extremely simple yet highly informative, providing an optimal balance for learning.</t>
+          <t>The movement is simple, direct, and perfectly captures the core concept without any unnecessary complexity, making it optimal for learning.</t>
         </is>
       </c>
       <c>
@@ -3079,7 +3079,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>This is a universally recognized gesture for an airplane in Western cultures, commonly used in childhood play.</t>
+          <t>Pretending to be an airplane by extending one's arms is a highly recognizable and universally understood gesture in Western cultures, often used in childhood play.</t>
         </is>
       </c>
       <c>
@@ -3098,7 +3098,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gross motor movements involved are very natural, simple, and effortless for learners to reproduce.</t>
+          <t>The gross motor movements of extending the arms and tilting the body are very natural, simple, and effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c>
-        <v>0.143</v>
+        <v>0.286</v>
       </c>
       <c>
         <v>1</v>
@@ -3323,17 +3323,17 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>Could also be interpreted as 'give' or 'offer' generally, rather than specifically a 'present'.</t>
-        </is>
-      </c>
-      <c>
-        <v>5</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>-1</v>
+          <t>The word 'present' can also mean 'current time' or 'to present (verb)', but the gesture clearly aligns with the noun meaning 'gift'.</t>
+        </is>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>0</v>
       </c>
       <c t="inlineStr">
         <is>
@@ -3342,17 +3342,17 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture clearly depicts the action of holding and offering a physical object, which strongly aligns with the concept of giving a present.</t>
-        </is>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>4</v>
-      </c>
-      <c>
-        <v>0</v>
+          <t>The gesture of holding an imaginary box and offering it forward perfectly mimics the action of giving a present.</t>
+        </is>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>5</v>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c t="inlineStr">
         <is>
@@ -3361,17 +3361,17 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The action of holding an imaginary box and extending the arms forward strongly evokes the physical experience of giving a gift.</t>
-        </is>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>3</v>
-      </c>
-      <c>
-        <v>0</v>
+          <t>Strongly evokes the physical sensation of holding an object with both hands and extending the arms to hand it over.</t>
+        </is>
+      </c>
+      <c>
+        <v>3</v>
+      </c>
+      <c>
+        <v>4</v>
+      </c>
+      <c>
+        <v>1</v>
       </c>
       <c t="inlineStr">
         <is>
@@ -3380,7 +3380,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is clear and involves both arms, but is relatively constrained and moderate in speed.</t>
+          <t>Clear, deliberate forward movement of both arms, making it visually distinct and easy to follow.</t>
         </is>
       </c>
       <c>
@@ -3418,7 +3418,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is simple, direct, and perfectly balances informativeness with ease of understanding.</t>
+          <t>The gesture is simple, intuitive, and directly conveys the meaning without unnecessary movements.</t>
         </is>
       </c>
       <c>
@@ -3437,7 +3437,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>Offering an object with both hands is a highly recognizable and common gesture for giving a present in Western cultures.</t>
+          <t>The action of offering an object with both hands is a universally recognized gesture for giving a gift in Western cultures.</t>
         </is>
       </c>
       <c>
@@ -3456,7 +3456,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is very natural, requires no special coordination, and is effortless to enact.</t>
+          <t>The movement is basic and requires no special coordination, making it effortless to copy.</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is a highly transparent and universally recognized pantomime of playing a guitar.</t>
+          <t>The gesture perfectly mimics the action of playing a guitar, providing a highly transparent visual representation of the target word.</t>
         </is>
       </c>
       <c>
@@ -3540,7 +3540,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture directly simulates the physical action, posture, and bodily experience of holding and strumming the instrument.</t>
+          <t>The gesture vividly simulates the physical interaction and bodily actions required to hold and strum a guitar.</t>
         </is>
       </c>
       <c>
@@ -3559,7 +3559,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The movement is clear and pronounced, involving both arms with a distinct, repetitive strumming action that draws attention.</t>
+          <t>The strumming motion and extended arm create a clear, pronounced, and easily noticeable movement.</t>
         </is>
       </c>
       <c>
@@ -3597,7 +3597,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is simple, intuitive, and perfectly captures the essence of the word without any unnecessary complexity.</t>
+          <t>The gesture is straightforward and perfectly captures the essence of the word without any unnecessary or confusing complexity.</t>
         </is>
       </c>
       <c>
@@ -3616,7 +3616,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The 'air guitar' gesture is highly familiar and widely used in Western culture to represent the instrument.</t>
+          <t>The 'air guitar' gesture is a highly familiar and universally recognized action in Western cultures.</t>
         </is>
       </c>
       <c>
@@ -3635,7 +3635,7 @@
       </c>
       <c t="inlineStr">
         <is>
-          <t>The gesture is very natural and effortless to enact, requiring no special physical skills or coordination.</t>
+          <t>The movements are simple, natural, and effortless for learners to reproduce.</t>
         </is>
       </c>
     </row>
@@ -24290,7 +24290,7 @@
         </is>
       </c>
       <c>
-        <v>0.672</v>
+        <v>0.657</v>
       </c>
     </row>
     <row r="7">
@@ -24300,7 +24300,7 @@
         </is>
       </c>
       <c>
-        <v>0.664</v>
+        <v>0.672</v>
       </c>
     </row>
     <row r="8">
@@ -24310,7 +24310,7 @@
         </is>
       </c>
       <c>
-        <v>0.418</v>
+        <v>0.425</v>
       </c>
     </row>
     <row r="9">
@@ -24320,7 +24320,7 @@
         </is>
       </c>
       <c>
-        <v>0.299</v>
+        <v>0.306</v>
       </c>
     </row>
     <row r="10">
@@ -24330,7 +24330,7 @@
         </is>
       </c>
       <c>
-        <v>0.343</v>
+        <v>0.328</v>
       </c>
     </row>
     <row r="11">
@@ -24340,7 +24340,7 @@
         </is>
       </c>
       <c>
-        <v>0.56</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Add concrete abstract dashboard view
</commit_message>
<xml_diff>
--- a/rating-results.xlsx
+++ b/rating-results.xlsx
@@ -24,6 +24,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>Concrete/abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Target word</t>
         </is>
       </c>
@@ -249,6 +254,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Traffic Light</t>
         </is>
       </c>
@@ -428,6 +438,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Trailer</t>
         </is>
       </c>
@@ -607,6 +622,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Balcony</t>
         </is>
       </c>
@@ -786,6 +806,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Ball</t>
         </is>
       </c>
@@ -965,6 +990,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bett</t>
         </is>
       </c>
@@ -1144,6 +1174,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Monitor</t>
         </is>
       </c>
@@ -1323,6 +1358,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Letter Box</t>
         </is>
       </c>
@@ -1502,6 +1542,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Ceiling</t>
         </is>
       </c>
@@ -1681,6 +1726,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Monument</t>
         </is>
       </c>
@@ -1860,6 +1910,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Entrance Ticket</t>
         </is>
       </c>
@@ -2039,6 +2094,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Thread</t>
         </is>
       </c>
@@ -2218,6 +2278,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bicycle</t>
         </is>
       </c>
@@ -2397,6 +2462,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Window</t>
         </is>
       </c>
@@ -2576,6 +2646,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Remote Control</t>
         </is>
       </c>
@@ -2755,6 +2830,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bottle</t>
         </is>
       </c>
@@ -2934,6 +3014,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Airplane</t>
         </is>
       </c>
@@ -3113,6 +3198,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
@@ -3292,6 +3382,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Present</t>
         </is>
       </c>
@@ -3471,6 +3566,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Guitar</t>
         </is>
       </c>
@@ -3650,6 +3750,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Purse</t>
         </is>
       </c>
@@ -3829,6 +3934,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Cable</t>
         </is>
       </c>
@@ -4008,6 +4118,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Camera</t>
         </is>
       </c>
@@ -4187,6 +4302,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Till</t>
         </is>
       </c>
@@ -4366,6 +4486,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Catalog</t>
         </is>
       </c>
@@ -4545,6 +4670,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Clothes</t>
         </is>
       </c>
@@ -4724,6 +4854,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Suitcase</t>
         </is>
       </c>
@@ -4903,6 +5038,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Machine</t>
         </is>
       </c>
@@ -5082,6 +5222,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Mask</t>
         </is>
       </c>
@@ -5261,6 +5406,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Paper</t>
         </is>
       </c>
@@ -5440,6 +5590,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tire</t>
         </is>
       </c>
@@ -5619,6 +5774,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Ring</t>
         </is>
       </c>
@@ -5798,6 +5958,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Backpack</t>
         </is>
       </c>
@@ -5977,6 +6142,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Collection</t>
         </is>
       </c>
@@ -6156,6 +6326,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Key</t>
         </is>
       </c>
@@ -6335,6 +6510,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Drawer</t>
         </is>
       </c>
@@ -6514,6 +6694,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Sunglasses</t>
         </is>
       </c>
@@ -6693,6 +6878,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Mirror</t>
         </is>
       </c>
@@ -6872,6 +7062,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tram</t>
         </is>
       </c>
@@ -7051,6 +7246,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Daily Newspaper</t>
         </is>
       </c>
@@ -7230,6 +7430,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Telephone</t>
         </is>
       </c>
@@ -7409,6 +7614,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Plate</t>
         </is>
       </c>
@@ -7588,6 +7798,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Carpet</t>
         </is>
       </c>
@@ -7767,6 +7982,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bandage</t>
         </is>
       </c>
@@ -7946,6 +8166,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tent</t>
         </is>
       </c>
@@ -8125,6 +8350,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Cigarette</t>
         </is>
       </c>
@@ -8304,6 +8534,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Cancellation</t>
         </is>
       </c>
@@ -8483,6 +8718,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Alternative</t>
         </is>
       </c>
@@ -8662,6 +8902,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Requirement</t>
         </is>
       </c>
@@ -8841,6 +9086,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Arrival</t>
         </is>
       </c>
@@ -9020,6 +9270,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Attention</t>
         </is>
       </c>
@@ -9199,6 +9454,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Effort</t>
         </is>
       </c>
@@ -9378,6 +9638,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>View</t>
         </is>
       </c>
@@ -9557,6 +9822,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Command</t>
         </is>
       </c>
@@ -9736,6 +10006,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Property</t>
         </is>
       </c>
@@ -9915,6 +10190,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Destination</t>
         </is>
       </c>
@@ -10094,6 +10374,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Plea</t>
         </is>
       </c>
@@ -10273,6 +10558,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Discipline</t>
         </is>
       </c>
@@ -10452,6 +10742,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Recommendation</t>
         </is>
       </c>
@@ -10631,6 +10926,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Thought</t>
         </is>
       </c>
@@ -10810,6 +11110,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Patience</t>
         </is>
       </c>
@@ -10989,6 +11294,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Indifference</t>
         </is>
       </c>
@@ -11168,6 +11478,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Information</t>
         </is>
       </c>
@@ -11347,6 +11662,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Correction</t>
         </is>
       </c>
@@ -11526,6 +11846,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Boredom</t>
         </is>
       </c>
@@ -11705,6 +12030,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Mentality</t>
         </is>
       </c>
@@ -11884,6 +12214,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Method</t>
         </is>
       </c>
@@ -12063,6 +12398,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bravery</t>
         </is>
       </c>
@@ -12242,6 +12582,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Partnership</t>
         </is>
       </c>
@@ -12421,6 +12766,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Consideration</t>
         </is>
       </c>
@@ -12600,6 +12950,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Sensation</t>
         </is>
       </c>
@@ -12779,6 +13134,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Style</t>
         </is>
       </c>
@@ -12958,6 +13318,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Talent</t>
         </is>
       </c>
@@ -13137,6 +13502,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Fact</t>
         </is>
       </c>
@@ -13316,6 +13686,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Participation</t>
         </is>
       </c>
@@ -13495,6 +13870,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tendency</t>
         </is>
       </c>
@@ -13674,6 +14054,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Theory</t>
         </is>
       </c>
@@ -13853,6 +14238,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Therapy</t>
         </is>
       </c>
@@ -14032,6 +14422,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tradition</t>
         </is>
       </c>
@@ -14211,6 +14606,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Triumph</t>
         </is>
       </c>
@@ -14390,6 +14790,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Exercise</t>
         </is>
       </c>
@@ -14569,6 +14974,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Innocence</t>
         </is>
       </c>
@@ -14748,6 +15158,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Change</t>
         </is>
       </c>
@@ -14927,6 +15342,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Sympathy</t>
         </is>
       </c>
@@ -15106,6 +15526,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Procedure</t>
         </is>
       </c>
@@ -15285,6 +15710,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Excuse</t>
         </is>
       </c>
@@ -15464,6 +15894,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Warning</t>
         </is>
       </c>
@@ -15643,6 +16078,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Wealth</t>
         </is>
       </c>
@@ -15822,6 +16262,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Benefaction</t>
         </is>
       </c>
@@ -16001,6 +16446,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Admission</t>
         </is>
       </c>
@@ -16180,6 +16630,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Purpose</t>
         </is>
       </c>
@@ -16359,6 +16814,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Zip</t>
         </is>
       </c>
@@ -16538,6 +16998,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Earring</t>
         </is>
       </c>
@@ -16717,6 +17182,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Peppermill</t>
         </is>
       </c>
@@ -16896,6 +17366,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Cup</t>
         </is>
       </c>
@@ -17075,6 +17550,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Broom</t>
         </is>
       </c>
@@ -17254,6 +17734,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Parsley</t>
         </is>
       </c>
@@ -17433,6 +17918,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Stairs</t>
         </is>
       </c>
@@ -17612,6 +18102,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Hair Dryer</t>
         </is>
       </c>
@@ -17791,6 +18286,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Watering Can</t>
         </is>
       </c>
@@ -17970,6 +18470,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tissue</t>
         </is>
       </c>
@@ -18149,6 +18654,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Soap</t>
         </is>
       </c>
@@ -18328,6 +18838,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Shelf</t>
         </is>
       </c>
@@ -18507,6 +19022,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Violin</t>
         </is>
       </c>
@@ -18686,6 +19206,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Stamp</t>
         </is>
       </c>
@@ -18865,6 +19390,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Thread</t>
         </is>
       </c>
@@ -19044,6 +19574,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Temple</t>
         </is>
       </c>
@@ -19223,6 +19758,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Chair</t>
         </is>
       </c>
@@ -19402,6 +19942,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Coffee</t>
         </is>
       </c>
@@ -19581,6 +20126,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Bridge</t>
         </is>
       </c>
@@ -19760,6 +20310,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Earth</t>
         </is>
       </c>
@@ -19939,6 +20494,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Flower</t>
         </is>
       </c>
@@ -20118,6 +20678,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Shampoo</t>
         </is>
       </c>
@@ -20297,6 +20862,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Jumper</t>
         </is>
       </c>
@@ -20476,6 +21046,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Dish Washing Liquid</t>
         </is>
       </c>
@@ -20655,6 +21230,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Pumpkin</t>
         </is>
       </c>
@@ -20834,6 +21414,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Eraser</t>
         </is>
       </c>
@@ -21013,6 +21598,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Stamp For Letter</t>
         </is>
       </c>
@@ -21192,6 +21782,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Flute</t>
         </is>
       </c>
@@ -21371,6 +21966,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Metal Sheet</t>
         </is>
       </c>
@@ -21550,6 +22150,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Towel</t>
         </is>
       </c>
@@ -21729,6 +22334,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Crutch</t>
         </is>
       </c>
@@ -21908,6 +22518,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Saw</t>
         </is>
       </c>
@@ -22087,6 +22702,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Perfume</t>
         </is>
       </c>
@@ -22266,6 +22886,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Tie</t>
         </is>
       </c>
@@ -22445,6 +23070,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Button</t>
         </is>
       </c>
@@ -22624,6 +23254,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Sponge</t>
         </is>
       </c>
@@ -22803,6 +23438,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Piece Of Paper</t>
         </is>
       </c>
@@ -22982,6 +23622,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Knife</t>
         </is>
       </c>
@@ -23161,6 +23806,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Wave</t>
         </is>
       </c>
@@ -23340,6 +23990,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Telephone</t>
         </is>
       </c>
@@ -23519,6 +24174,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Mirror</t>
         </is>
       </c>
@@ -23698,6 +24358,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Remote Control</t>
         </is>
       </c>
@@ -23877,6 +24542,11 @@
       </c>
       <c t="inlineStr">
         <is>
+          <t>concrete</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
           <t>Banana</t>
         </is>
       </c>
@@ -24052,6 +24722,11 @@
       <c t="inlineStr">
         <is>
           <t>object</t>
+        </is>
+      </c>
+      <c t="inlineStr">
+        <is>
+          <t>concrete</t>
         </is>
       </c>
       <c t="inlineStr">

</xml_diff>